<commit_message>
data: Actualización automática de reportes (2026-07-06 14:03)
</commit_message>
<xml_diff>
--- a/VENTAS_MENSUALES/MAYO_CORREGIDO_RESULTADO.xlsx
+++ b/VENTAS_MENSUALES/MAYO_CORREGIDO_RESULTADO.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G53"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -435,22 +435,22 @@
         <v>DARINKA UREÐA CASILLAS</v>
       </c>
       <c r="B2">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="C2">
         <v>4</v>
       </c>
       <c r="D2">
-        <v>174469.28677022</v>
+        <v>41370.92</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>2339.79</v>
       </c>
       <c r="G2">
-        <v>174469.28677022</v>
+        <v>43710.71</v>
       </c>
     </row>
     <row r="3">
@@ -464,7 +464,7 @@
         <v>2</v>
       </c>
       <c r="D3">
-        <v>71108.24392390001</v>
+        <v>24572.42</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -473,7 +473,7 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>71108.24392390001</v>
+        <v>24572.42</v>
       </c>
     </row>
     <row r="4">
@@ -487,7 +487,7 @@
         <v>1</v>
       </c>
       <c r="D4">
-        <v>22666.414424632498</v>
+        <v>5250.63</v>
       </c>
       <c r="E4">
         <v>0.5</v>
@@ -496,7 +496,7 @@
         <v>2724.89</v>
       </c>
       <c r="G4">
-        <v>25391.304424632497</v>
+        <v>7975.52</v>
       </c>
     </row>
     <row r="5">
@@ -625,7 +625,7 @@
         <v>2</v>
       </c>
       <c r="D10">
-        <v>36662.53761354</v>
+        <v>36647.08</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -634,7 +634,7 @@
         <v>0</v>
       </c>
       <c r="G10">
-        <v>36662.53761354</v>
+        <v>36647.08</v>
       </c>
     </row>
     <row r="11">
@@ -832,7 +832,7 @@
         <v>1</v>
       </c>
       <c r="D19">
-        <v>11237.05142364</v>
+        <v>1562.88</v>
       </c>
       <c r="E19">
         <v>0.5</v>
@@ -841,7 +841,7 @@
         <v>56328.79</v>
       </c>
       <c r="G19">
-        <v>67565.84142364</v>
+        <v>57891.67</v>
       </c>
     </row>
     <row r="20">
@@ -1488,9 +1488,147 @@
         <v>6304.46</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>ANA LAURA CONTRERAS IÑIGUEZ</v>
+      </c>
+      <c r="B48">
+        <v>1.5</v>
+      </c>
+      <c r="C48">
+        <v>1</v>
+      </c>
+      <c r="D48">
+        <v>22666.414424632498</v>
+      </c>
+      <c r="E48">
+        <v>0.5</v>
+      </c>
+      <c r="F48">
+        <v>2724.89</v>
+      </c>
+      <c r="G48">
+        <v>25391.304424632497</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>DARINKA UREÑA CASILLAS</v>
+      </c>
+      <c r="B49">
+        <v>3</v>
+      </c>
+      <c r="C49">
+        <v>3</v>
+      </c>
+      <c r="D49">
+        <v>140824.51208795</v>
+      </c>
+      <c r="E49">
+        <v>0</v>
+      </c>
+      <c r="F49">
+        <v>0</v>
+      </c>
+      <c r="G49">
+        <v>140824.51208795</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>DESIREE DE LA PEÑA OROZCO</v>
+      </c>
+      <c r="B50">
+        <v>2</v>
+      </c>
+      <c r="C50">
+        <v>2</v>
+      </c>
+      <c r="D50">
+        <v>71108.24392390001</v>
+      </c>
+      <c r="E50">
+        <v>0</v>
+      </c>
+      <c r="F50">
+        <v>0</v>
+      </c>
+      <c r="G50">
+        <v>71108.24392390001</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>GABRIELA CASTAÑEDA SALAZAR</v>
+      </c>
+      <c r="B51">
+        <v>2</v>
+      </c>
+      <c r="C51">
+        <v>2</v>
+      </c>
+      <c r="D51">
+        <v>36662.53761354</v>
+      </c>
+      <c r="E51">
+        <v>0</v>
+      </c>
+      <c r="F51">
+        <v>0</v>
+      </c>
+      <c r="G51">
+        <v>36662.53761354</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>PAULINA LIZBETH SOTO MUÑIZ</v>
+      </c>
+      <c r="B52">
+        <v>1.5</v>
+      </c>
+      <c r="C52">
+        <v>1</v>
+      </c>
+      <c r="D52">
+        <v>11237.05142364</v>
+      </c>
+      <c r="E52">
+        <v>0.5</v>
+      </c>
+      <c r="F52">
+        <v>56328.79</v>
+      </c>
+      <c r="G52">
+        <v>67565.84142364</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>COLUMNA</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Columna12</v>
+      </c>
+      <c r="C53">
+        <v>0</v>
+      </c>
+      <c r="D53">
+        <v>0</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Columna12</v>
+      </c>
+      <c r="F53" t="str">
+        <v>Columna3</v>
+      </c>
+      <c r="G53" t="str">
+        <v>Columna3</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G53"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>